<commit_message>
actualiza Excel, detecta horarios anómalos y renueva logo
</commit_message>
<xml_diff>
--- a/data/actual/GUIAS X SEMANA Y HORARIOS.xlsx
+++ b/data/actual/GUIAS X SEMANA Y HORARIOS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30524"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcovarrubia\OneDrive - Universidad Tecnologica del Peru\LABORATORIOS\2. HORARIOS SEMANALES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4527F761-E43F-4144-AAB5-48A739D0A8FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BC6A6D9-EE9D-4639-9049-17B251B7419F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30" yWindow="30" windowWidth="20460" windowHeight="10770" firstSheet="8" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7481,7 +7481,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:31" ht="14.45" hidden="1">
@@ -10181,7 +10181,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:32" ht="14.45" hidden="1">
@@ -15669,7 +15669,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:32" ht="14.45" hidden="1">
@@ -21221,7 +21221,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:32" ht="14.45" hidden="1">
@@ -26621,7 +26621,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:31" ht="14.45" hidden="1">
@@ -29278,7 +29278,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:31" ht="14.45" hidden="1">
@@ -32839,7 +32839,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:31" ht="14.45" hidden="1">
@@ -35491,7 +35491,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:32" ht="14.45" hidden="1">
@@ -40542,7 +40542,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:31" ht="14.45" hidden="1">
@@ -43254,7 +43254,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:32" ht="14.45" hidden="1">
@@ -48730,7 +48730,6 @@
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="6.85546875" customWidth="1"/>
-    <col min="2" max="2" width="11.42578125" customWidth="1"/>
     <col min="4" max="4" width="11.42578125" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="0" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" hidden="1" customWidth="1"/>
@@ -48816,7 +48815,7 @@
       <c r="AC2" s="26"/>
       <c r="AD2" s="15">
         <f ca="1">TODAY()</f>
-        <v>46292</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="3" spans="2:31" ht="14.45" hidden="1">

</xml_diff>